<commit_message>
deleted feature sum_of_points, cause it seems to be some leekage of data, and it is not relevant for future model
</commit_message>
<xml_diff>
--- a/predictions_table.xlsx
+++ b/predictions_table.xlsx
@@ -496,10 +496,10 @@
         <v>1</v>
       </c>
       <c r="G2" t="n">
-        <v>7.24</v>
+        <v>7.11</v>
       </c>
       <c r="H2" t="n">
-        <v>6.24</v>
+        <v>6.11</v>
       </c>
     </row>
     <row r="3">
@@ -528,10 +528,10 @@
         <v>2</v>
       </c>
       <c r="G3" t="n">
-        <v>10.65</v>
+        <v>10.89</v>
       </c>
       <c r="H3" t="n">
-        <v>8.65</v>
+        <v>8.890000000000001</v>
       </c>
     </row>
     <row r="4">
@@ -560,10 +560,10 @@
         <v>3</v>
       </c>
       <c r="G4" t="n">
-        <v>5.09</v>
+        <v>5.04</v>
       </c>
       <c r="H4" t="n">
-        <v>2.09</v>
+        <v>2.04</v>
       </c>
     </row>
     <row r="5">
@@ -592,10 +592,10 @@
         <v>4</v>
       </c>
       <c r="G5" t="n">
-        <v>3.56</v>
+        <v>3.28</v>
       </c>
       <c r="H5" t="n">
-        <v>-0.4399999999999999</v>
+        <v>-0.7200000000000002</v>
       </c>
     </row>
     <row r="6">
@@ -624,10 +624,10 @@
         <v>5</v>
       </c>
       <c r="G6" t="n">
-        <v>9.4</v>
+        <v>9.24</v>
       </c>
       <c r="H6" t="n">
-        <v>4.4</v>
+        <v>4.24</v>
       </c>
     </row>
     <row r="7">
@@ -656,10 +656,10 @@
         <v>6</v>
       </c>
       <c r="G7" t="n">
-        <v>9.710000000000001</v>
+        <v>9.58</v>
       </c>
       <c r="H7" t="n">
-        <v>3.710000000000001</v>
+        <v>3.58</v>
       </c>
     </row>
     <row r="8">
@@ -688,10 +688,10 @@
         <v>7</v>
       </c>
       <c r="G8" t="n">
-        <v>7.54</v>
+        <v>7.45</v>
       </c>
       <c r="H8" t="n">
-        <v>0.54</v>
+        <v>0.4500000000000002</v>
       </c>
     </row>
     <row r="9">
@@ -720,10 +720,10 @@
         <v>8</v>
       </c>
       <c r="G9" t="n">
-        <v>7.64</v>
+        <v>7.61</v>
       </c>
       <c r="H9" t="n">
-        <v>-0.3600000000000003</v>
+        <v>-0.3899999999999997</v>
       </c>
     </row>
     <row r="10">
@@ -752,10 +752,10 @@
         <v>9</v>
       </c>
       <c r="G10" t="n">
-        <v>8.07</v>
+        <v>8.09</v>
       </c>
       <c r="H10" t="n">
-        <v>-0.9299999999999997</v>
+        <v>-0.9100000000000001</v>
       </c>
     </row>
     <row r="11">
@@ -784,10 +784,10 @@
         <v>10</v>
       </c>
       <c r="G11" t="n">
-        <v>11.62</v>
+        <v>11.6</v>
       </c>
       <c r="H11" t="n">
-        <v>1.619999999999999</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="12">
@@ -816,10 +816,10 @@
         <v>11</v>
       </c>
       <c r="G12" t="n">
-        <v>13.16</v>
+        <v>13.12</v>
       </c>
       <c r="H12" t="n">
-        <v>2.16</v>
+        <v>2.119999999999999</v>
       </c>
     </row>
     <row r="13">
@@ -848,10 +848,10 @@
         <v>12</v>
       </c>
       <c r="G13" t="n">
-        <v>11.94</v>
+        <v>11.97</v>
       </c>
       <c r="H13" t="n">
-        <v>-0.0600000000000005</v>
+        <v>-0.02999999999999936</v>
       </c>
     </row>
     <row r="14">
@@ -880,10 +880,10 @@
         <v>13</v>
       </c>
       <c r="G14" t="n">
-        <v>10.17</v>
+        <v>10.12</v>
       </c>
       <c r="H14" t="n">
-        <v>-2.83</v>
+        <v>-2.880000000000001</v>
       </c>
     </row>
     <row r="15">
@@ -912,10 +912,10 @@
         <v>14</v>
       </c>
       <c r="G15" t="n">
-        <v>15.34</v>
+        <v>15.36</v>
       </c>
       <c r="H15" t="n">
-        <v>1.34</v>
+        <v>1.359999999999999</v>
       </c>
     </row>
     <row r="16">
@@ -944,10 +944,10 @@
         <v>15</v>
       </c>
       <c r="G16" t="n">
-        <v>14.75</v>
+        <v>14.62</v>
       </c>
       <c r="H16" t="n">
-        <v>-0.25</v>
+        <v>-0.3800000000000008</v>
       </c>
     </row>
     <row r="17">
@@ -976,10 +976,10 @@
         <v>16</v>
       </c>
       <c r="G17" t="n">
-        <v>14.28</v>
+        <v>14.27</v>
       </c>
       <c r="H17" t="n">
-        <v>-1.720000000000001</v>
+        <v>-1.73</v>
       </c>
     </row>
     <row r="18">
@@ -1008,10 +1008,10 @@
         <v>17</v>
       </c>
       <c r="G18" t="n">
-        <v>17.26</v>
+        <v>17.29</v>
       </c>
       <c r="H18" t="n">
-        <v>0.2600000000000016</v>
+        <v>0.2899999999999991</v>
       </c>
     </row>
     <row r="19">
@@ -1040,10 +1040,10 @@
         <v>18</v>
       </c>
       <c r="G19" t="n">
-        <v>17.99</v>
+        <v>18.02</v>
       </c>
       <c r="H19" t="n">
-        <v>-0.01000000000000156</v>
+        <v>0.01999999999999957</v>
       </c>
     </row>
     <row r="20">
@@ -1072,10 +1072,10 @@
         <v>19</v>
       </c>
       <c r="G20" t="n">
-        <v>15.83</v>
+        <v>15.85</v>
       </c>
       <c r="H20" t="n">
-        <v>-3.17</v>
+        <v>-3.15</v>
       </c>
     </row>
     <row r="21">
@@ -1104,10 +1104,10 @@
         <v>20</v>
       </c>
       <c r="G21" t="n">
-        <v>8.18</v>
+        <v>8.16</v>
       </c>
       <c r="H21" t="n">
-        <v>-11.82</v>
+        <v>-11.84</v>
       </c>
     </row>
     <row r="22">
@@ -1136,10 +1136,10 @@
         <v>1</v>
       </c>
       <c r="G22" t="n">
-        <v>2.6</v>
+        <v>2.73</v>
       </c>
       <c r="H22" t="n">
-        <v>1.6</v>
+        <v>1.73</v>
       </c>
     </row>
     <row r="23">
@@ -1168,10 +1168,10 @@
         <v>2</v>
       </c>
       <c r="G23" t="n">
-        <v>8.130000000000001</v>
+        <v>7.7</v>
       </c>
       <c r="H23" t="n">
-        <v>6.130000000000001</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="24">
@@ -1200,10 +1200,10 @@
         <v>3</v>
       </c>
       <c r="G24" t="n">
-        <v>4.08</v>
+        <v>4.19</v>
       </c>
       <c r="H24" t="n">
-        <v>1.08</v>
+        <v>1.19</v>
       </c>
     </row>
     <row r="25">
@@ -1232,10 +1232,10 @@
         <v>4</v>
       </c>
       <c r="G25" t="n">
-        <v>4.27</v>
+        <v>4.56</v>
       </c>
       <c r="H25" t="n">
-        <v>0.2699999999999996</v>
+        <v>0.5599999999999996</v>
       </c>
     </row>
     <row r="26">
@@ -1264,10 +1264,10 @@
         <v>5</v>
       </c>
       <c r="G26" t="n">
-        <v>6.08</v>
+        <v>6.1</v>
       </c>
       <c r="H26" t="n">
-        <v>1.08</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="27">
@@ -1296,10 +1296,10 @@
         <v>6</v>
       </c>
       <c r="G27" t="n">
-        <v>9.279999999999999</v>
+        <v>9.43</v>
       </c>
       <c r="H27" t="n">
-        <v>3.279999999999999</v>
+        <v>3.43</v>
       </c>
     </row>
     <row r="28">
@@ -1328,10 +1328,10 @@
         <v>7</v>
       </c>
       <c r="G28" t="n">
-        <v>9.98</v>
+        <v>10.02</v>
       </c>
       <c r="H28" t="n">
-        <v>2.98</v>
+        <v>3.02</v>
       </c>
     </row>
     <row r="29">
@@ -1360,10 +1360,10 @@
         <v>8</v>
       </c>
       <c r="G29" t="n">
-        <v>7.37</v>
+        <v>7.36</v>
       </c>
       <c r="H29" t="n">
-        <v>-0.6299999999999999</v>
+        <v>-0.6399999999999997</v>
       </c>
     </row>
     <row r="30">
@@ -1392,10 +1392,10 @@
         <v>9</v>
       </c>
       <c r="G30" t="n">
-        <v>12.15</v>
+        <v>12.24</v>
       </c>
       <c r="H30" t="n">
-        <v>3.15</v>
+        <v>3.24</v>
       </c>
     </row>
     <row r="31">
@@ -1424,10 +1424,10 @@
         <v>10</v>
       </c>
       <c r="G31" t="n">
-        <v>12.7</v>
+        <v>12.71</v>
       </c>
       <c r="H31" t="n">
-        <v>2.699999999999999</v>
+        <v>2.710000000000001</v>
       </c>
     </row>
     <row r="32">
@@ -1456,10 +1456,10 @@
         <v>11</v>
       </c>
       <c r="G32" t="n">
-        <v>11.2</v>
+        <v>11.22</v>
       </c>
       <c r="H32" t="n">
-        <v>0.1999999999999993</v>
+        <v>0.2200000000000006</v>
       </c>
     </row>
     <row r="33">
@@ -1488,10 +1488,10 @@
         <v>12</v>
       </c>
       <c r="G33" t="n">
-        <v>14.12</v>
+        <v>14.14</v>
       </c>
       <c r="H33" t="n">
-        <v>2.119999999999999</v>
+        <v>2.140000000000001</v>
       </c>
     </row>
     <row r="34">
@@ -1520,10 +1520,10 @@
         <v>13</v>
       </c>
       <c r="G34" t="n">
-        <v>10.98</v>
+        <v>11</v>
       </c>
       <c r="H34" t="n">
-        <v>-2.02</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="35">
@@ -1552,10 +1552,10 @@
         <v>14</v>
       </c>
       <c r="G35" t="n">
-        <v>8.09</v>
+        <v>7.96</v>
       </c>
       <c r="H35" t="n">
-        <v>-5.91</v>
+        <v>-6.04</v>
       </c>
     </row>
     <row r="36">
@@ -1584,10 +1584,10 @@
         <v>15</v>
       </c>
       <c r="G36" t="n">
-        <v>12.44</v>
+        <v>12.41</v>
       </c>
       <c r="H36" t="n">
-        <v>-2.56</v>
+        <v>-2.59</v>
       </c>
     </row>
     <row r="37">
@@ -1616,10 +1616,10 @@
         <v>16</v>
       </c>
       <c r="G37" t="n">
-        <v>15.55</v>
+        <v>15.47</v>
       </c>
       <c r="H37" t="n">
-        <v>-0.4499999999999993</v>
+        <v>-0.5299999999999994</v>
       </c>
     </row>
     <row r="38">
@@ -1648,10 +1648,10 @@
         <v>17</v>
       </c>
       <c r="G38" t="n">
-        <v>11.76</v>
+        <v>11.5</v>
       </c>
       <c r="H38" t="n">
-        <v>-5.24</v>
+        <v>-5.5</v>
       </c>
     </row>
     <row r="39">
@@ -1680,10 +1680,10 @@
         <v>18</v>
       </c>
       <c r="G39" t="n">
-        <v>17.18</v>
+        <v>17.23</v>
       </c>
       <c r="H39" t="n">
-        <v>-0.8200000000000003</v>
+        <v>-0.7699999999999996</v>
       </c>
     </row>
     <row r="40">
@@ -1712,10 +1712,10 @@
         <v>19</v>
       </c>
       <c r="G40" t="n">
-        <v>12.71</v>
+        <v>12.59</v>
       </c>
       <c r="H40" t="n">
-        <v>-6.289999999999999</v>
+        <v>-6.41</v>
       </c>
     </row>
     <row r="41">
@@ -1744,10 +1744,10 @@
         <v>20</v>
       </c>
       <c r="G41" t="n">
-        <v>16.78</v>
+        <v>16.69</v>
       </c>
       <c r="H41" t="n">
-        <v>-3.219999999999999</v>
+        <v>-3.309999999999999</v>
       </c>
     </row>
     <row r="42">
@@ -1776,10 +1776,10 @@
         <v>1</v>
       </c>
       <c r="G42" t="n">
-        <v>2.04</v>
+        <v>1.98</v>
       </c>
       <c r="H42" t="n">
-        <v>1.04</v>
+        <v>0.98</v>
       </c>
     </row>
     <row r="43">
@@ -1808,10 +1808,10 @@
         <v>2</v>
       </c>
       <c r="G43" t="n">
-        <v>9.77</v>
+        <v>9.68</v>
       </c>
       <c r="H43" t="n">
-        <v>7.77</v>
+        <v>7.68</v>
       </c>
     </row>
     <row r="44">
@@ -1840,10 +1840,10 @@
         <v>3</v>
       </c>
       <c r="G44" t="n">
-        <v>8.31</v>
+        <v>8.369999999999999</v>
       </c>
       <c r="H44" t="n">
-        <v>5.31</v>
+        <v>5.369999999999999</v>
       </c>
     </row>
     <row r="45">
@@ -1872,10 +1872,10 @@
         <v>4</v>
       </c>
       <c r="G45" t="n">
-        <v>4.28</v>
+        <v>4.21</v>
       </c>
       <c r="H45" t="n">
-        <v>0.2800000000000002</v>
+        <v>0.21</v>
       </c>
     </row>
     <row r="46">
@@ -1904,10 +1904,10 @@
         <v>5</v>
       </c>
       <c r="G46" t="n">
-        <v>7.8</v>
+        <v>7.9</v>
       </c>
       <c r="H46" t="n">
-        <v>2.8</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="47">
@@ -1936,10 +1936,10 @@
         <v>6</v>
       </c>
       <c r="G47" t="n">
-        <v>6.01</v>
+        <v>6.09</v>
       </c>
       <c r="H47" t="n">
-        <v>0.009999999999999787</v>
+        <v>0.08999999999999986</v>
       </c>
     </row>
     <row r="48">
@@ -1968,10 +1968,10 @@
         <v>7</v>
       </c>
       <c r="G48" t="n">
-        <v>8.859999999999999</v>
+        <v>8.9</v>
       </c>
       <c r="H48" t="n">
-        <v>1.859999999999999</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="49">
@@ -2000,10 +2000,10 @@
         <v>8</v>
       </c>
       <c r="G49" t="n">
-        <v>9.25</v>
+        <v>9.26</v>
       </c>
       <c r="H49" t="n">
-        <v>1.25</v>
+        <v>1.26</v>
       </c>
     </row>
     <row r="50">
@@ -2032,10 +2032,10 @@
         <v>9</v>
       </c>
       <c r="G50" t="n">
-        <v>12.21</v>
+        <v>12.13</v>
       </c>
       <c r="H50" t="n">
-        <v>3.210000000000001</v>
+        <v>3.130000000000001</v>
       </c>
     </row>
     <row r="51">
@@ -2096,10 +2096,10 @@
         <v>11</v>
       </c>
       <c r="G52" t="n">
-        <v>13.51</v>
+        <v>13.52</v>
       </c>
       <c r="H52" t="n">
-        <v>2.51</v>
+        <v>2.52</v>
       </c>
     </row>
     <row r="53">
@@ -2128,10 +2128,10 @@
         <v>12</v>
       </c>
       <c r="G53" t="n">
-        <v>15.36</v>
+        <v>15.39</v>
       </c>
       <c r="H53" t="n">
-        <v>3.359999999999999</v>
+        <v>3.390000000000001</v>
       </c>
     </row>
     <row r="54">
@@ -2160,10 +2160,10 @@
         <v>13</v>
       </c>
       <c r="G54" t="n">
-        <v>11.12</v>
+        <v>11.03</v>
       </c>
       <c r="H54" t="n">
-        <v>-1.880000000000001</v>
+        <v>-1.970000000000001</v>
       </c>
     </row>
     <row r="55">
@@ -2192,10 +2192,10 @@
         <v>14</v>
       </c>
       <c r="G55" t="n">
-        <v>14.81</v>
+        <v>14.83</v>
       </c>
       <c r="H55" t="n">
-        <v>0.8100000000000005</v>
+        <v>0.8300000000000001</v>
       </c>
     </row>
     <row r="56">
@@ -2224,10 +2224,10 @@
         <v>15</v>
       </c>
       <c r="G56" t="n">
-        <v>13.8</v>
+        <v>13.84</v>
       </c>
       <c r="H56" t="n">
-        <v>-1.199999999999999</v>
+        <v>-1.16</v>
       </c>
     </row>
     <row r="57">
@@ -2256,10 +2256,10 @@
         <v>16</v>
       </c>
       <c r="G57" t="n">
-        <v>8.529999999999999</v>
+        <v>8.49</v>
       </c>
       <c r="H57" t="n">
-        <v>-7.470000000000001</v>
+        <v>-7.51</v>
       </c>
     </row>
     <row r="58">
@@ -2288,10 +2288,10 @@
         <v>17</v>
       </c>
       <c r="G58" t="n">
-        <v>12.25</v>
+        <v>12.33</v>
       </c>
       <c r="H58" t="n">
-        <v>-4.75</v>
+        <v>-4.67</v>
       </c>
     </row>
     <row r="59">
@@ -2320,10 +2320,10 @@
         <v>18</v>
       </c>
       <c r="G59" t="n">
-        <v>15.4</v>
+        <v>15.06</v>
       </c>
       <c r="H59" t="n">
-        <v>-2.6</v>
+        <v>-2.94</v>
       </c>
     </row>
     <row r="60">
@@ -2352,10 +2352,10 @@
         <v>19</v>
       </c>
       <c r="G60" t="n">
-        <v>9.99</v>
+        <v>9.85</v>
       </c>
       <c r="H60" t="n">
-        <v>-9.01</v>
+        <v>-9.15</v>
       </c>
     </row>
     <row r="61">
@@ -2384,10 +2384,10 @@
         <v>20</v>
       </c>
       <c r="G61" t="n">
-        <v>19.52</v>
+        <v>19.58</v>
       </c>
       <c r="H61" t="n">
-        <v>-0.4800000000000004</v>
+        <v>-0.4200000000000017</v>
       </c>
     </row>
     <row r="62">
@@ -2416,10 +2416,10 @@
         <v>1</v>
       </c>
       <c r="G62" t="n">
-        <v>1.94</v>
+        <v>1.88</v>
       </c>
       <c r="H62" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.8799999999999999</v>
       </c>
     </row>
     <row r="63">
@@ -2448,10 +2448,10 @@
         <v>2</v>
       </c>
       <c r="G63" t="n">
-        <v>2.59</v>
+        <v>2.84</v>
       </c>
       <c r="H63" t="n">
-        <v>0.5899999999999999</v>
+        <v>0.8399999999999999</v>
       </c>
     </row>
     <row r="64">
@@ -2480,10 +2480,10 @@
         <v>3</v>
       </c>
       <c r="G64" t="n">
-        <v>3.44</v>
+        <v>3.47</v>
       </c>
       <c r="H64" t="n">
-        <v>0.4399999999999999</v>
+        <v>0.4700000000000002</v>
       </c>
     </row>
     <row r="65">
@@ -2512,10 +2512,10 @@
         <v>4</v>
       </c>
       <c r="G65" t="n">
-        <v>4.66</v>
+        <v>4.65</v>
       </c>
       <c r="H65" t="n">
-        <v>0.6600000000000001</v>
+        <v>0.6500000000000004</v>
       </c>
     </row>
     <row r="66">
@@ -2544,10 +2544,10 @@
         <v>5</v>
       </c>
       <c r="G66" t="n">
-        <v>5.61</v>
+        <v>5.59</v>
       </c>
       <c r="H66" t="n">
-        <v>0.6100000000000003</v>
+        <v>0.5899999999999999</v>
       </c>
     </row>
     <row r="67">
@@ -2576,10 +2576,10 @@
         <v>6</v>
       </c>
       <c r="G67" t="n">
-        <v>6.54</v>
+        <v>6.53</v>
       </c>
       <c r="H67" t="n">
-        <v>0.54</v>
+        <v>0.5300000000000002</v>
       </c>
     </row>
     <row r="68">
@@ -2608,10 +2608,10 @@
         <v>7</v>
       </c>
       <c r="G68" t="n">
-        <v>6.93</v>
+        <v>6.96</v>
       </c>
       <c r="H68" t="n">
-        <v>-0.07000000000000028</v>
+        <v>-0.04000000000000004</v>
       </c>
     </row>
     <row r="69">
@@ -2640,10 +2640,10 @@
         <v>8</v>
       </c>
       <c r="G69" t="n">
-        <v>7.9</v>
+        <v>7.95</v>
       </c>
       <c r="H69" t="n">
-        <v>-0.09999999999999964</v>
+        <v>-0.04999999999999982</v>
       </c>
     </row>
     <row r="70">
@@ -2672,10 +2672,10 @@
         <v>9</v>
       </c>
       <c r="G70" t="n">
-        <v>10.47</v>
+        <v>10.01</v>
       </c>
       <c r="H70" t="n">
-        <v>1.470000000000001</v>
+        <v>1.01</v>
       </c>
     </row>
     <row r="71">
@@ -2704,10 +2704,10 @@
         <v>10</v>
       </c>
       <c r="G71" t="n">
-        <v>10.01</v>
+        <v>10.06</v>
       </c>
       <c r="H71" t="n">
-        <v>0.009999999999999787</v>
+        <v>0.0600000000000005</v>
       </c>
     </row>
     <row r="72">
@@ -2736,10 +2736,10 @@
         <v>11</v>
       </c>
       <c r="G72" t="n">
-        <v>11.41</v>
+        <v>11.31</v>
       </c>
       <c r="H72" t="n">
-        <v>0.4100000000000001</v>
+        <v>0.3100000000000005</v>
       </c>
     </row>
     <row r="73">
@@ -2800,10 +2800,10 @@
         <v>13</v>
       </c>
       <c r="G74" t="n">
-        <v>13.42</v>
+        <v>13.34</v>
       </c>
       <c r="H74" t="n">
-        <v>0.4199999999999999</v>
+        <v>0.3399999999999999</v>
       </c>
     </row>
     <row r="75">
@@ -2832,10 +2832,10 @@
         <v>14</v>
       </c>
       <c r="G75" t="n">
-        <v>14.33</v>
+        <v>14.35</v>
       </c>
       <c r="H75" t="n">
-        <v>0.3300000000000001</v>
+        <v>0.3499999999999996</v>
       </c>
     </row>
     <row r="76">
@@ -2864,10 +2864,10 @@
         <v>15</v>
       </c>
       <c r="G76" t="n">
-        <v>14.83</v>
+        <v>14.8</v>
       </c>
       <c r="H76" t="n">
-        <v>-0.1699999999999999</v>
+        <v>-0.1999999999999993</v>
       </c>
     </row>
     <row r="77">
@@ -2896,10 +2896,10 @@
         <v>16</v>
       </c>
       <c r="G77" t="n">
-        <v>16.25</v>
+        <v>16.28</v>
       </c>
       <c r="H77" t="n">
-        <v>0.25</v>
+        <v>0.2800000000000011</v>
       </c>
     </row>
     <row r="78">
@@ -2928,10 +2928,10 @@
         <v>17</v>
       </c>
       <c r="G78" t="n">
-        <v>17.45</v>
+        <v>17.47</v>
       </c>
       <c r="H78" t="n">
-        <v>0.4499999999999993</v>
+        <v>0.4699999999999989</v>
       </c>
     </row>
     <row r="79">
@@ -2960,10 +2960,10 @@
         <v>18</v>
       </c>
       <c r="G79" t="n">
-        <v>17.68</v>
+        <v>17.65</v>
       </c>
       <c r="H79" t="n">
-        <v>-0.3200000000000003</v>
+        <v>-0.3500000000000014</v>
       </c>
     </row>
     <row r="80">
@@ -2992,10 +2992,10 @@
         <v>19</v>
       </c>
       <c r="G80" t="n">
-        <v>19.21</v>
+        <v>19.22</v>
       </c>
       <c r="H80" t="n">
-        <v>0.2100000000000009</v>
+        <v>0.2199999999999989</v>
       </c>
     </row>
     <row r="81">
@@ -3024,10 +3024,10 @@
         <v>20</v>
       </c>
       <c r="G81" t="n">
-        <v>19.39</v>
+        <v>19.31</v>
       </c>
       <c r="H81" t="n">
-        <v>-0.6099999999999994</v>
+        <v>-0.6900000000000013</v>
       </c>
     </row>
     <row r="82">
@@ -3056,10 +3056,10 @@
         <v>1</v>
       </c>
       <c r="G82" t="n">
-        <v>1.94</v>
+        <v>1.9</v>
       </c>
       <c r="H82" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.8999999999999999</v>
       </c>
     </row>
     <row r="83">
@@ -3088,10 +3088,10 @@
         <v>2</v>
       </c>
       <c r="G83" t="n">
-        <v>3</v>
+        <v>3.19</v>
       </c>
       <c r="H83" t="n">
-        <v>1</v>
+        <v>1.19</v>
       </c>
     </row>
     <row r="84">
@@ -3152,10 +3152,10 @@
         <v>4</v>
       </c>
       <c r="G85" t="n">
-        <v>4.27</v>
+        <v>4.56</v>
       </c>
       <c r="H85" t="n">
-        <v>0.2699999999999996</v>
+        <v>0.5599999999999996</v>
       </c>
     </row>
     <row r="86">
@@ -3184,10 +3184,10 @@
         <v>5</v>
       </c>
       <c r="G86" t="n">
-        <v>9.880000000000001</v>
+        <v>9.789999999999999</v>
       </c>
       <c r="H86" t="n">
-        <v>4.880000000000001</v>
+        <v>4.789999999999999</v>
       </c>
     </row>
     <row r="87">
@@ -3216,10 +3216,10 @@
         <v>6</v>
       </c>
       <c r="G87" t="n">
-        <v>7.71</v>
+        <v>7.49</v>
       </c>
       <c r="H87" t="n">
-        <v>1.71</v>
+        <v>1.49</v>
       </c>
     </row>
     <row r="88">
@@ -3248,10 +3248,10 @@
         <v>7</v>
       </c>
       <c r="G88" t="n">
-        <v>10</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="H88" t="n">
-        <v>3</v>
+        <v>2.970000000000001</v>
       </c>
     </row>
     <row r="89">
@@ -3280,10 +3280,10 @@
         <v>8</v>
       </c>
       <c r="G89" t="n">
-        <v>7.93</v>
+        <v>7.71</v>
       </c>
       <c r="H89" t="n">
-        <v>-0.07000000000000028</v>
+        <v>-0.29</v>
       </c>
     </row>
     <row r="90">
@@ -3312,10 +3312,10 @@
         <v>9</v>
       </c>
       <c r="G90" t="n">
-        <v>9.550000000000001</v>
+        <v>9.56</v>
       </c>
       <c r="H90" t="n">
-        <v>0.5500000000000007</v>
+        <v>0.5600000000000005</v>
       </c>
     </row>
     <row r="91">
@@ -3344,10 +3344,10 @@
         <v>10</v>
       </c>
       <c r="G91" t="n">
-        <v>9.539999999999999</v>
+        <v>9.609999999999999</v>
       </c>
       <c r="H91" t="n">
-        <v>-0.4600000000000009</v>
+        <v>-0.3900000000000006</v>
       </c>
     </row>
     <row r="92">
@@ -3376,10 +3376,10 @@
         <v>11</v>
       </c>
       <c r="G92" t="n">
-        <v>11.02</v>
+        <v>11.03</v>
       </c>
       <c r="H92" t="n">
-        <v>0.01999999999999957</v>
+        <v>0.02999999999999936</v>
       </c>
     </row>
     <row r="93">
@@ -3408,10 +3408,10 @@
         <v>12</v>
       </c>
       <c r="G93" t="n">
-        <v>11.33</v>
+        <v>11.35</v>
       </c>
       <c r="H93" t="n">
-        <v>-0.6699999999999999</v>
+        <v>-0.6500000000000004</v>
       </c>
     </row>
     <row r="94">
@@ -3440,10 +3440,10 @@
         <v>13</v>
       </c>
       <c r="G94" t="n">
-        <v>12.23</v>
+        <v>12.26</v>
       </c>
       <c r="H94" t="n">
-        <v>-0.7699999999999996</v>
+        <v>-0.7400000000000002</v>
       </c>
     </row>
     <row r="95">
@@ -3472,10 +3472,10 @@
         <v>14</v>
       </c>
       <c r="G95" t="n">
-        <v>12.54</v>
+        <v>12.47</v>
       </c>
       <c r="H95" t="n">
-        <v>-1.460000000000001</v>
+        <v>-1.529999999999999</v>
       </c>
     </row>
     <row r="96">
@@ -3504,10 +3504,10 @@
         <v>15</v>
       </c>
       <c r="G96" t="n">
-        <v>15.34</v>
+        <v>15.36</v>
       </c>
       <c r="H96" t="n">
-        <v>0.3399999999999999</v>
+        <v>0.3599999999999994</v>
       </c>
     </row>
     <row r="97">
@@ -3536,10 +3536,10 @@
         <v>16</v>
       </c>
       <c r="G97" t="n">
-        <v>12.21</v>
+        <v>12.18</v>
       </c>
       <c r="H97" t="n">
-        <v>-3.789999999999999</v>
+        <v>-3.82</v>
       </c>
     </row>
     <row r="98">
@@ -3568,10 +3568,10 @@
         <v>17</v>
       </c>
       <c r="G98" t="n">
-        <v>17.35</v>
+        <v>17.38</v>
       </c>
       <c r="H98" t="n">
-        <v>0.3500000000000014</v>
+        <v>0.379999999999999</v>
       </c>
     </row>
     <row r="99">
@@ -3600,10 +3600,10 @@
         <v>18</v>
       </c>
       <c r="G99" t="n">
-        <v>14.19</v>
+        <v>14.16</v>
       </c>
       <c r="H99" t="n">
-        <v>-3.81</v>
+        <v>-3.84</v>
       </c>
     </row>
     <row r="100">
@@ -3632,10 +3632,10 @@
         <v>19</v>
       </c>
       <c r="G100" t="n">
-        <v>16.76</v>
+        <v>16.57</v>
       </c>
       <c r="H100" t="n">
-        <v>-2.239999999999998</v>
+        <v>-2.43</v>
       </c>
     </row>
     <row r="101">
@@ -3664,10 +3664,10 @@
         <v>20</v>
       </c>
       <c r="G101" t="n">
-        <v>15.52</v>
+        <v>15.54</v>
       </c>
       <c r="H101" t="n">
-        <v>-4.48</v>
+        <v>-4.460000000000001</v>
       </c>
     </row>
     <row r="102">
@@ -3696,10 +3696,10 @@
         <v>1</v>
       </c>
       <c r="G102" t="n">
-        <v>3.34</v>
+        <v>3.48</v>
       </c>
       <c r="H102" t="n">
-        <v>2.34</v>
+        <v>2.48</v>
       </c>
     </row>
     <row r="103">
@@ -3728,10 +3728,10 @@
         <v>2</v>
       </c>
       <c r="G103" t="n">
-        <v>6.71</v>
+        <v>6.93</v>
       </c>
       <c r="H103" t="n">
-        <v>4.71</v>
+        <v>4.93</v>
       </c>
     </row>
     <row r="104">
@@ -3760,10 +3760,10 @@
         <v>3</v>
       </c>
       <c r="G104" t="n">
-        <v>5.02</v>
+        <v>5.07</v>
       </c>
       <c r="H104" t="n">
-        <v>2.02</v>
+        <v>2.07</v>
       </c>
     </row>
     <row r="105">
@@ -3792,10 +3792,10 @@
         <v>4</v>
       </c>
       <c r="G105" t="n">
-        <v>4.74</v>
+        <v>4.78</v>
       </c>
       <c r="H105" t="n">
-        <v>0.7400000000000002</v>
+        <v>0.7800000000000002</v>
       </c>
     </row>
     <row r="106">
@@ -3824,10 +3824,10 @@
         <v>5</v>
       </c>
       <c r="G106" t="n">
-        <v>8.66</v>
+        <v>8.380000000000001</v>
       </c>
       <c r="H106" t="n">
-        <v>3.66</v>
+        <v>3.380000000000001</v>
       </c>
     </row>
     <row r="107">
@@ -3856,10 +3856,10 @@
         <v>6</v>
       </c>
       <c r="G107" t="n">
-        <v>7.51</v>
+        <v>7.13</v>
       </c>
       <c r="H107" t="n">
-        <v>1.51</v>
+        <v>1.13</v>
       </c>
     </row>
     <row r="108">
@@ -3888,10 +3888,10 @@
         <v>7</v>
       </c>
       <c r="G108" t="n">
-        <v>6.06</v>
+        <v>6.08</v>
       </c>
       <c r="H108" t="n">
-        <v>-0.9400000000000004</v>
+        <v>-0.9199999999999999</v>
       </c>
     </row>
     <row r="109">
@@ -3920,10 +3920,10 @@
         <v>8</v>
       </c>
       <c r="G109" t="n">
-        <v>6.05</v>
+        <v>5.92</v>
       </c>
       <c r="H109" t="n">
-        <v>-1.95</v>
+        <v>-2.08</v>
       </c>
     </row>
     <row r="110">
@@ -3952,10 +3952,10 @@
         <v>9</v>
       </c>
       <c r="G110" t="n">
-        <v>8.199999999999999</v>
+        <v>8.32</v>
       </c>
       <c r="H110" t="n">
-        <v>-0.8000000000000007</v>
+        <v>-0.6799999999999997</v>
       </c>
     </row>
     <row r="111">
@@ -3984,10 +3984,10 @@
         <v>10</v>
       </c>
       <c r="G111" t="n">
-        <v>14.65</v>
+        <v>14.69</v>
       </c>
       <c r="H111" t="n">
-        <v>4.65</v>
+        <v>4.69</v>
       </c>
     </row>
     <row r="112">
@@ -4016,10 +4016,10 @@
         <v>11</v>
       </c>
       <c r="G112" t="n">
-        <v>12.02</v>
+        <v>11.87</v>
       </c>
       <c r="H112" t="n">
-        <v>1.02</v>
+        <v>0.8699999999999992</v>
       </c>
     </row>
     <row r="113">
@@ -4080,10 +4080,10 @@
         <v>13</v>
       </c>
       <c r="G114" t="n">
-        <v>10.71</v>
+        <v>10.91</v>
       </c>
       <c r="H114" t="n">
-        <v>-2.289999999999999</v>
+        <v>-2.09</v>
       </c>
     </row>
     <row r="115">
@@ -4112,10 +4112,10 @@
         <v>14</v>
       </c>
       <c r="G115" t="n">
-        <v>13.89</v>
+        <v>13.8</v>
       </c>
       <c r="H115" t="n">
-        <v>-0.1099999999999994</v>
+        <v>-0.1999999999999993</v>
       </c>
     </row>
     <row r="116">
@@ -4144,10 +4144,10 @@
         <v>15</v>
       </c>
       <c r="G116" t="n">
-        <v>14.47</v>
+        <v>14.43</v>
       </c>
       <c r="H116" t="n">
-        <v>-0.5299999999999994</v>
+        <v>-0.5700000000000003</v>
       </c>
     </row>
     <row r="117">
@@ -4176,10 +4176,10 @@
         <v>16</v>
       </c>
       <c r="G117" t="n">
-        <v>11.58</v>
+        <v>11.55</v>
       </c>
       <c r="H117" t="n">
-        <v>-4.42</v>
+        <v>-4.449999999999999</v>
       </c>
     </row>
     <row r="118">
@@ -4208,10 +4208,10 @@
         <v>17</v>
       </c>
       <c r="G118" t="n">
-        <v>16.5</v>
+        <v>16.55</v>
       </c>
       <c r="H118" t="n">
-        <v>-0.5</v>
+        <v>-0.4499999999999993</v>
       </c>
     </row>
     <row r="119">
@@ -4240,10 +4240,10 @@
         <v>18</v>
       </c>
       <c r="G119" t="n">
-        <v>14.71</v>
+        <v>14.73</v>
       </c>
       <c r="H119" t="n">
-        <v>-3.289999999999999</v>
+        <v>-3.27</v>
       </c>
     </row>
     <row r="120">
@@ -4304,10 +4304,10 @@
         <v>20</v>
       </c>
       <c r="G121" t="n">
-        <v>18.47</v>
+        <v>18.48</v>
       </c>
       <c r="H121" t="n">
-        <v>-1.530000000000001</v>
+        <v>-1.52</v>
       </c>
     </row>
     <row r="122">
@@ -4336,10 +4336,10 @@
         <v>1</v>
       </c>
       <c r="G122" t="n">
-        <v>2.39</v>
+        <v>2.23</v>
       </c>
       <c r="H122" t="n">
-        <v>1.39</v>
+        <v>1.23</v>
       </c>
     </row>
     <row r="123">
@@ -4432,10 +4432,10 @@
         <v>4</v>
       </c>
       <c r="G125" t="n">
-        <v>9.27</v>
+        <v>9.4</v>
       </c>
       <c r="H125" t="n">
-        <v>5.27</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="126">
@@ -4464,10 +4464,10 @@
         <v>5</v>
       </c>
       <c r="G126" t="n">
-        <v>9.08</v>
+        <v>9.09</v>
       </c>
       <c r="H126" t="n">
-        <v>4.08</v>
+        <v>4.09</v>
       </c>
     </row>
     <row r="127">
@@ -4496,10 +4496,10 @@
         <v>6</v>
       </c>
       <c r="G127" t="n">
-        <v>8.73</v>
+        <v>8.720000000000001</v>
       </c>
       <c r="H127" t="n">
-        <v>2.73</v>
+        <v>2.720000000000001</v>
       </c>
     </row>
     <row r="128">
@@ -4528,10 +4528,10 @@
         <v>7</v>
       </c>
       <c r="G128" t="n">
-        <v>7.47</v>
+        <v>7.66</v>
       </c>
       <c r="H128" t="n">
-        <v>0.4699999999999998</v>
+        <v>0.6600000000000001</v>
       </c>
     </row>
     <row r="129">
@@ -4560,10 +4560,10 @@
         <v>8</v>
       </c>
       <c r="G129" t="n">
-        <v>10.5</v>
+        <v>10.3</v>
       </c>
       <c r="H129" t="n">
-        <v>2.5</v>
+        <v>2.300000000000001</v>
       </c>
     </row>
     <row r="130">
@@ -4592,10 +4592,10 @@
         <v>9</v>
       </c>
       <c r="G130" t="n">
-        <v>7.03</v>
+        <v>6.82</v>
       </c>
       <c r="H130" t="n">
-        <v>-1.97</v>
+        <v>-2.18</v>
       </c>
     </row>
     <row r="131">
@@ -4624,10 +4624,10 @@
         <v>10</v>
       </c>
       <c r="G131" t="n">
-        <v>11.8</v>
+        <v>11.82</v>
       </c>
       <c r="H131" t="n">
-        <v>1.800000000000001</v>
+        <v>1.82</v>
       </c>
     </row>
     <row r="132">
@@ -4656,10 +4656,10 @@
         <v>11</v>
       </c>
       <c r="G132" t="n">
-        <v>14.57</v>
+        <v>14.59</v>
       </c>
       <c r="H132" t="n">
-        <v>3.57</v>
+        <v>3.59</v>
       </c>
     </row>
     <row r="133">
@@ -4688,10 +4688,10 @@
         <v>12</v>
       </c>
       <c r="G133" t="n">
-        <v>10.7</v>
+        <v>10.73</v>
       </c>
       <c r="H133" t="n">
-        <v>-1.300000000000001</v>
+        <v>-1.27</v>
       </c>
     </row>
     <row r="134">
@@ -4720,10 +4720,10 @@
         <v>13</v>
       </c>
       <c r="G134" t="n">
-        <v>8.85</v>
+        <v>8.9</v>
       </c>
       <c r="H134" t="n">
-        <v>-4.15</v>
+        <v>-4.1</v>
       </c>
     </row>
     <row r="135">
@@ -4752,10 +4752,10 @@
         <v>14</v>
       </c>
       <c r="G135" t="n">
-        <v>15.52</v>
+        <v>15.54</v>
       </c>
       <c r="H135" t="n">
-        <v>1.52</v>
+        <v>1.539999999999999</v>
       </c>
     </row>
     <row r="136">
@@ -4784,10 +4784,10 @@
         <v>15</v>
       </c>
       <c r="G136" t="n">
-        <v>14.37</v>
+        <v>14.39</v>
       </c>
       <c r="H136" t="n">
-        <v>-0.6300000000000008</v>
+        <v>-0.6099999999999994</v>
       </c>
     </row>
     <row r="137">
@@ -4816,10 +4816,10 @@
         <v>16</v>
       </c>
       <c r="G137" t="n">
-        <v>13.01</v>
+        <v>13.05</v>
       </c>
       <c r="H137" t="n">
-        <v>-2.99</v>
+        <v>-2.949999999999999</v>
       </c>
     </row>
     <row r="138">
@@ -4848,10 +4848,10 @@
         <v>17</v>
       </c>
       <c r="G138" t="n">
-        <v>13.81</v>
+        <v>13.79</v>
       </c>
       <c r="H138" t="n">
-        <v>-3.19</v>
+        <v>-3.210000000000001</v>
       </c>
     </row>
     <row r="139">
@@ -4880,10 +4880,10 @@
         <v>18</v>
       </c>
       <c r="G139" t="n">
-        <v>14.71</v>
+        <v>14.72</v>
       </c>
       <c r="H139" t="n">
-        <v>-3.289999999999999</v>
+        <v>-3.279999999999999</v>
       </c>
     </row>
     <row r="140">
@@ -4912,10 +4912,10 @@
         <v>19</v>
       </c>
       <c r="G140" t="n">
-        <v>15.42</v>
+        <v>15.4</v>
       </c>
       <c r="H140" t="n">
-        <v>-3.58</v>
+        <v>-3.6</v>
       </c>
     </row>
     <row r="141">

</xml_diff>